<commit_message>
Template v2; report lists columns filled from the data but not used by the model yet
</commit_message>
<xml_diff>
--- a/schema/Schema_Template_EMPTY.xlsx
+++ b/schema/Schema_Template_EMPTY.xlsx
@@ -1689,7 +1689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6560,7 +6560,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>read but not used</t>
+          <t>source data, not in model yet</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>ignored</t>
+          <t>in the source data; not used by the model yet (staffing_factor_per_machine is used)</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -6595,7 +6595,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>not used</t>
+          <t>not used yet</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>read but not used</t>
+          <t>source data, not in model yet</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>ignored; availability comes from MTBF_hours / MTTR_min</t>
+          <t>in the source data; not used by the model yet; open decision whether to apply it (availability comes from MTBF_hours / MTTR_min for now)</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
-          <t>not used</t>
+          <t>open decision</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>read but not used</t>
+          <t>source data, not in model yet</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>ignored if present; cleaning time is inside setup_time_min</t>
+          <t>in the source data; not used by the model yet (cleaning time is inside setup_time_min)</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
@@ -6689,7 +6689,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>not used</t>
+          <t>not used yet</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>read but not used</t>
+          <t>source data, not in model yet</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>ignored if present</t>
+          <t>in the source data; not used by the model yet</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
@@ -6736,430 +6736,7 @@
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B109" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>num_replications</t>
-        </is>
-      </c>
-      <c r="E109" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F109" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>ignored; runs are started by hand</t>
-        </is>
-      </c>
-      <c r="H109" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I109" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B110" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C110" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D110" s="4" t="inlineStr">
-        <is>
-          <t>random_seed</t>
-        </is>
-      </c>
-      <c r="E110" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F110" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>ignored; each run takes its own seed</t>
-        </is>
-      </c>
-      <c r="H110" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I110" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>interarrival_dist</t>
-        </is>
-      </c>
-      <c r="E111" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F111" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>ignored</t>
-        </is>
-      </c>
-      <c r="H111" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I111" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C112" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>interarrival_param</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F112" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G112" s="2" t="inlineStr">
-        <is>
-          <t>ignored</t>
-        </is>
-      </c>
-      <c r="H112" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I112" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>queue_discipline</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G113" s="2" t="inlineStr">
-        <is>
-          <t>ignored; replaced by queue_rule</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I113" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C114" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D114" s="4" t="inlineStr">
-        <is>
-          <t>workers_optional</t>
-        </is>
-      </c>
-      <c r="E114" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>ignored; Workers sheet presence decides</t>
-        </is>
-      </c>
-      <c r="H114" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I114" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>kpi_machine_util</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="inlineStr">
-        <is>
-          <t>ignored</t>
-        </is>
-      </c>
-      <c r="H115" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I115" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D116" s="4" t="inlineStr">
-        <is>
-          <t>kpi_worker_util</t>
-        </is>
-      </c>
-      <c r="E116" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F116" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>ignored</t>
-        </is>
-      </c>
-      <c r="H116" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I116" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>read but not used</t>
-        </is>
-      </c>
-      <c r="C117" s="4" t="inlineStr">
-        <is>
-          <t>Config</t>
-        </is>
-      </c>
-      <c r="D117" s="4" t="inlineStr">
-        <is>
-          <t>kpi_throughput_time</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="inlineStr">
-        <is>
-          <t>Config key</t>
-        </is>
-      </c>
-      <c r="F117" s="4" t="inlineStr">
-        <is>
-          <t>optional</t>
-        </is>
-      </c>
-      <c r="G117" s="2" t="inlineStr">
-        <is>
-          <t>ignored</t>
-        </is>
-      </c>
-      <c r="H117" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I117" s="4" t="inlineStr">
-        <is>
-          <t>not used</t>
+          <t>not used yet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use the Dictionary column when_module_on: needed columns of a filled module sheet count as required; report shows module and role
</commit_message>
<xml_diff>
--- a/schema/Schema_Template_EMPTY.xlsx
+++ b/schema/Schema_Template_EMPTY.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -480,197 +480,204 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A missing optional sheet, or one with no data, turns that module off. A blank cell takes the default listed in Dictionary. A cell reading TODO means the source data has no value; the model treats it like a blank.</t>
+          <t>Dictionary column 'when_module_on' says, for each column, its role once its module is on: switch (turns it on), needed (must be filled) or optional (blank takes the default).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Columns marked 'pos N' are read by position: do not move or delete them. Columns marked 'header name' may be absent or anywhere.</t>
+          <t>A missing optional sheet, or one with no data, turns that module off. A blank cell takes the default listed in Dictionary. A cell reading TODO means the source data has no value; the model treats it like a blank.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Columns marked 'pos N' are read by position: do not move or delete them. Columns marked 'header name' may be absent or anywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Extra sheets (README, Overview, Dictionary) are ignored by the model.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Modules</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M0 Core flow (required). Status: tested. Switch: always on.</t>
+          <t>Modules</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Products are released as lots and follow their Routing step by step. Each step needs one machine unit of the named resource group for the setup time plus cycle time x pieces, then the transport time to the next step.</t>
+          <t>M0 Core flow (required). Status: tested. Switch: always on.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>M1 Calendar (optional). Status: tested. Switch: Shifts sheet (required in practice); ResourceShiftCalendar sheet present.</t>
+          <t xml:space="preserve">    Products are released as lots and follow their Routing step by step. Each step needs one machine unit of the named resource group for the setup time plus cycle time x pieces, then the transport time to the next step.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Shifts say when resources work; ResourceShiftCalendar gives each machine or worker its shift pattern, with dates and a capacity multiplier. A step starts only when its machine (and worker) is on shift; warmup_min adds a start-up time per machine.</t>
+          <t>M1 Calendar (optional). Status: tested. Switch: Shifts sheet (required in practice); ResourceShiftCalendar sheet present.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>M2 Workforce (optional). Status: tested, effect recorded. Switch: Workers sheet present.</t>
+          <t xml:space="preserve">    Shifts say when resources work; ResourceShiftCalendar gives each machine or worker its shift pattern, with dates and a capacity multiplier. A step starts only when its machine (and worker) is on shift; warmup_min adds a start-up time per machine.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Workers with a shift, skills per resource group and a limit on parallel machines. A step starts only when a qualified worker is free, for the setup only or for the whole step (worker_needed_during). Worker choice: first fit or least utilised; efficiency factor optional. Off: machines are limited by capacity and shifts only.</t>
+          <t>M2 Workforce (optional). Status: tested, effect recorded. Switch: Workers sheet present.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>M3 Routing alternatives (optional). Status: tested. Switch: Alternatives sheet present.</t>
+          <t xml:space="preserve">    Workers with a shift, skills per resource group and a limit on parallel machines. A step starts only when a qualified worker is free, for the setup only or for the whole step (worker_needed_during). Worker choice: first fit or least utilised; efficiency factor optional. Off: machines are limited by capacity and shifts only.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Which machines of a group a step may use, in priority order, with a run-time factor per machine. Off: every machine of the group qualifies.</t>
+          <t>M3 Routing alternatives (optional). Status: tested. Switch: Alternatives sheet present.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>M4 Demand and batching (optional). Status: tested. Switch: Config demand_mode = order, batch_mode = on.</t>
+          <t xml:space="preserve">    Which machines of a group a step may use, in priority order, with a run-time factor per machine. Off: every machine of the group qualifies.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Lot mode: each product releases a lot at random with mean gap arrival_interval_min. Order mode: each arrival releases order_quantity x arrival_interval_min / order_window_min pieces, cut into lots. Batch mode: lots of one product share one machine run up to batch_size; a batch waits at most batch_overhead_min x batch_wait_margin. Off: lot mode, no batching.</t>
+          <t>M4 Demand and batching (optional). Status: tested. Switch: Config demand_mode = order, batch_mode = on.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>M5 Order replay (optional). Status: tested. Switch: Config demand_mode = replay.</t>
+          <t xml:space="preserve">    Lot mode: each product releases a lot at random with mean gap arrival_interval_min. Order mode: each arrival releases order_quantity x arrival_interval_min / order_window_min pieces, cut into lots. Batch mode: lots of one product share one machine run up to batch_size; a batch waits at most batch_overhead_min x batch_wait_margin. Off: lot mode, no batching.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Releases exactly the rows of the Orders sheet at release_min, with due date, priority and order type; queues can rank by priority, then release time. Reports lateness and on-time rate. Off: arrivals come from Products.</t>
+          <t>M5 Order replay (optional). Status: tested. Switch: Config demand_mode = replay.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>M6 Setup matrix (optional). Status: tested. Switch: SetupMatrix sheet present.</t>
+          <t xml:space="preserve">    Releases exactly the rows of the Orders sheet at release_min, with due date, priority and order type; queues can rank by priority, then release time. Reports lateness and on-time rate. Off: arrivals come from Products.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Setup time depends on the change of setup family on the machine (from family to family, per resource group). Off: the Routing setup_time_min is paid on every lot.</t>
+          <t>M6 Setup matrix (optional). Status: tested. Switch: SetupMatrix sheet present.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>M7 Reliability (optional). Status: tested. Switch: Machines MTBF_hours &gt; 0.</t>
+          <t xml:space="preserve">    Setup time depends on the change of setup family on the machine (from family to family, per resource group). Off: the Routing setup_time_min is paid on every lot.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Machines fail at random (exponential time between failures, mean MTBF_hours, counted only in shift time) and are repaired in exactly MTTR_min; a failure during a step adds the repair time to that step. Off: no breakdowns.</t>
+          <t>M7 Reliability (optional). Status: tested. Switch: Machines MTBF_hours &gt; 0.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>M8 Material (optional). Status: tested. Switch: Config material_mode = boards.</t>
+          <t xml:space="preserve">    Machines fail at random (exponential time between failures, mean MTBF_hours, counted only in shift time) and are repaired in exactly MTTR_min; a failure during a step adds the repair time to that step. Off: no breakdowns.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Before a lot starts, its components (BOM) are taken from stock (Inventory). Components the model makes itself must be in stock, so the lot waits for them without holding a machine; bought materials are counted, not limiting. Off: material is unlimited.</t>
+          <t>M8 Material (optional). Status: tested. Switch: Config material_mode = boards.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>M9 Quality (optional). Status: tested. Switch: Config quality_mode = yield.</t>
+          <t xml:space="preserve">    Before a lot starts, its components (BOM) are taken from stock (Inventory). Components the model makes itself must be in stock, so the lot waits for them without holding a machine; bought materials are counted, not limiting. Off: material is unlimited.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    yield_pct per step; failed pieces are scrapped or reworked once (scrap_or_rework). Scrapped pieces of an order get make-up lots, at most 5 per order. Off: 100 % yield.</t>
+          <t>M9 Quality (optional). Status: tested. Switch: Config quality_mode = yield.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>M10 Cost (optional). Status: tested. Switch: Machines cost_per_hour &gt; 0.</t>
+          <t xml:space="preserve">    yield_pct per step; failed pieces are scrapped or reworked once (scrap_or_rework). Scrapped pieces of an order get make-up lots, at most 5 per order. Off: 100 % yield.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Output only, no effect on the flow: machine cost per busy and per shift hour, labour cost, cost per good piece. Off: no cost rows.</t>
+          <t>M10 Cost (optional). Status: tested. Switch: Machines cost_per_hour &gt; 0.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>M11 Scenarios (optional). Status: built, not yet tested (test planned Mon 2026-10-26). Switch: Experiment parameter scenario_id names rows of the Scenarios sheet.</t>
+          <t xml:space="preserve">    Output only, no effect on the flow: machine cost per busy and per shift hour, labour cost, cost per good piece. Off: no cost rows.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
+        <is>
+          <t>M11 Scenarios (optional). Status: built, not yet tested (test planned Mon 2026-10-26). Switch: Experiment parameter scenario_id names rows of the Scenarios sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">    A scenario is a few rows, not a new file: each row changes the base factory in memory (set a value, scale a column, copy a machine / worker / product with its linked rows, remove one). The Experiment parameter scenario_id picks the rows; empty = base factory. The base sheets stay unchanged, and a wrong row stops the run with a message.</t>
         </is>
@@ -1689,7 +1696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1698,16 +1705,17 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dictionary: one row per sheet and column. Source: model reader code (ExcelSchemaReader, SimConfig).</t>
+          <t>Dictionary: one row per sheet and column. Source: model reader code (ExcelSchemaReader, SimConfig). when_module_on: switch = turns the module on; needed = must be filled once the module is on; optional = blank takes the default.</t>
         </is>
       </c>
     </row>
@@ -1744,15 +1752,20 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>when_module_on</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>if_blank_or_missing</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>switch</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -1791,15 +1804,20 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>row skipped</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -1838,15 +1856,20 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -1885,15 +1908,20 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1 piece)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1 piece</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -1932,15 +1960,20 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>row skipped / DEFAULT 0</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -1979,15 +2012,20 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>row skipped / DEFAULT 0</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2026,15 +2064,20 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2073,15 +2116,20 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>empty or unknown group: run REJECTED at startup ('Routing references groups with no machines'); a Machines row without a group is skipped with a warning</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2120,15 +2168,20 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>needed (blank = 0 minutes)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2167,15 +2220,20 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2214,15 +2272,20 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2261,15 +2324,20 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
           <t>row skipped / empty text</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2308,15 +2376,20 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
           <t>row skipped / empty text</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2355,15 +2428,20 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
           <t>row skipped / empty text</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2402,15 +2480,20 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2449,15 +2532,20 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 10,080 / 1,440 min)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 10,080 / 1,440 min</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2496,15 +2584,20 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 10,080 / 1,440 min)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 10,080 / 1,440 min</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2543,15 +2636,20 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT "not_set")</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT "not_set"</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>always on</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2590,15 +2688,20 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
+          <t>switch (a filled Shifts sheet)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2637,15 +2740,20 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2684,15 +2792,20 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2731,15 +2844,20 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2778,15 +2896,20 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2825,15 +2948,20 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2872,15 +3000,20 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
           <t>no Shifts sheet: every machine has no shift, so an autonomous run is REJECTED (the default shift must exist in Shifts); a worker run is rejected when a worker names an unknown shift. In practice Shifts is required</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2919,15 +3052,20 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -2966,15 +3104,20 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3013,15 +3156,20 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3060,15 +3208,20 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3107,15 +3260,20 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3154,15 +3312,20 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: flat Shifts for all; valid_to empty = open end; multiplier DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3201,15 +3364,20 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="J33" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3248,15 +3416,20 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
+          <t>needed (runs without workers)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
           <t>autonomous run: machines without a calendar row get this shift (logged as an assumption); key empty or unknown shift: run REJECTED. Worker run: not used, a machine without its own shift follows its qualified workers' shifts</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3295,15 +3468,20 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
           <t>empty: valid_from / valid_to cannot be dated</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>Shifts sheet (required in practice); ResourceShiftCalendar sheet present</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -3342,15 +3520,20 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
+          <t>switch (a filled Workers sheet)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: OFF, machines limited by capacity and shifts only</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="J36" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3389,15 +3572,20 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: OFF, machines limited by capacity and shifts only</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="J37" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3436,15 +3624,20 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
+          <t>needed (must exist in Shifts)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: OFF, machines limited by capacity and shifts only</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="J38" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3483,15 +3676,20 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1.0)</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="J39" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3530,15 +3728,20 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="J40" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3577,15 +3780,20 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
           <t>skill_level DEFAULT 1</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="I41" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="J41" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3624,15 +3832,20 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
           <t>skill_level DEFAULT 1</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
+      <c r="J42" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3671,15 +3884,20 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1)</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
           <t>skill_level DEFAULT 1</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="J43" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3718,15 +3936,20 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT yes)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT yes</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="J44" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3765,15 +3988,20 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT yes)</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT yes</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="I45" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I45" s="4" t="inlineStr">
+      <c r="J45" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3812,15 +4040,20 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT yes)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT yes</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3859,15 +4092,20 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Workers max_parallel_machines; value DEFAULT 1</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I47" s="4" t="inlineStr">
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3906,15 +4144,20 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Workers max_parallel_machines; value DEFAULT 1</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I48" s="4" t="inlineStr">
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -3953,15 +4196,20 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Workers max_parallel_machines; value DEFAULT 1</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr">
+      <c r="I49" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr">
+      <c r="J49" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4000,15 +4248,20 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="I50" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I50" s="4" t="inlineStr">
+      <c r="J50" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4047,15 +4300,20 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1.0)</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4094,15 +4352,20 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT whole_step)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT whole_step; "none" read as setup</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr">
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I52" s="4" t="inlineStr">
+      <c r="J52" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4141,15 +4404,20 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT FIRST_FIT)</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT FIRST_FIT (or LEAST_UTILIZED)</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr">
+      <c r="I53" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I53" s="4" t="inlineStr">
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4188,15 +4456,20 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT false)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT false</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr">
+      <c r="I54" s="4" t="inlineStr">
         <is>
           <t>Workers sheet present</t>
         </is>
       </c>
-      <c r="I54" s="4" t="inlineStr">
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>tested, effect recorded</t>
         </is>
@@ -4235,15 +4508,20 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
+          <t>switch (a filled Alternatives sheet)</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: every machine of the group qualifies</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
+      <c r="I55" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4282,15 +4560,20 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: every machine of the group qualifies</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
+      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4329,15 +4612,20 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: every machine of the group qualifies</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I57" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4376,15 +4664,20 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: every machine of the group qualifies</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr">
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I58" s="4" t="inlineStr">
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4423,15 +4716,20 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 99)</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 99</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr">
+      <c r="I59" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="J59" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4470,15 +4768,20 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1.0)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1.0</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr">
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>Alternatives sheet present</t>
         </is>
       </c>
-      <c r="I60" s="4" t="inlineStr">
+      <c r="J60" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4517,15 +4820,20 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
+          <t>needed (order mode)</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1</t>
         </is>
       </c>
-      <c r="H61" s="4" t="inlineStr">
+      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I61" s="4" t="inlineStr">
+      <c r="J61" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4564,15 +4872,20 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
+          <t>needed (order mode)</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0 (then a synthetic mean of 20,000 min)</t>
         </is>
       </c>
-      <c r="H62" s="4" t="inlineStr">
+      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I62" s="4" t="inlineStr">
+      <c r="J62" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4611,15 +4924,20 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
+          <t>needed (batching)</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1</t>
         </is>
       </c>
-      <c r="H63" s="4" t="inlineStr">
+      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I63" s="4" t="inlineStr">
+      <c r="J63" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4658,15 +4976,20 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr">
+      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I64" s="4" t="inlineStr">
+      <c r="J64" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4705,15 +5028,20 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
+          <t>switch (order = M4, replay = M5)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT lot</t>
         </is>
       </c>
-      <c r="H65" s="4" t="inlineStr">
+      <c r="I65" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I65" s="4" t="inlineStr">
+      <c r="J65" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4752,15 +5080,20 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
+          <t>needed (order mode)</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr">
+      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I66" s="4" t="inlineStr">
+      <c r="J66" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4799,15 +5132,20 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
+          <t>switch (on = batching)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT off</t>
         </is>
       </c>
-      <c r="H67" s="4" t="inlineStr">
+      <c r="I67" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I67" s="4" t="inlineStr">
+      <c r="J67" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4846,15 +5184,20 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1.0 / 1,440 min)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1.0 / 1,440 min</t>
         </is>
       </c>
-      <c r="H68" s="4" t="inlineStr">
+      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I68" s="4" t="inlineStr">
+      <c r="J68" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4893,15 +5236,20 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 1.0 / 1,440 min)</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 1.0 / 1,440 min</t>
         </is>
       </c>
-      <c r="H69" s="4" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = order, batch_mode = on</t>
         </is>
       </c>
-      <c r="I69" s="4" t="inlineStr">
+      <c r="J69" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4940,15 +5288,20 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: OFF, arrivals from Products</t>
         </is>
       </c>
-      <c r="H70" s="4" t="inlineStr">
+      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I70" s="4" t="inlineStr">
+      <c r="J70" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -4987,15 +5340,20 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: OFF, arrivals from Products</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
+      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I71" s="4" t="inlineStr">
+      <c r="J71" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5034,15 +5392,20 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H72" s="4" t="inlineStr">
+      <c r="I72" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I72" s="4" t="inlineStr">
+      <c r="J72" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5081,15 +5444,20 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
+          <t>needed (run rejected without it)</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT -1 = missing: replay run REJECTED (release_min &lt; 0, or due_min before release_min). Both are required in replay mode</t>
         </is>
       </c>
-      <c r="H73" s="4" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I73" s="4" t="inlineStr">
+      <c r="J73" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5128,15 +5496,20 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
+          <t>needed (run rejected without it)</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT -1 = missing: replay run REJECTED (release_min &lt; 0, or due_min before release_min). Both are required in replay mode</t>
         </is>
       </c>
-      <c r="H74" s="4" t="inlineStr">
+      <c r="I74" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I74" s="4" t="inlineStr">
+      <c r="J74" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5175,15 +5548,20 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 99)</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 99</t>
         </is>
       </c>
-      <c r="H75" s="4" t="inlineStr">
+      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I75" s="4" t="inlineStr">
+      <c r="J75" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5222,15 +5600,20 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H76" s="4" t="inlineStr">
+      <c r="I76" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I76" s="4" t="inlineStr">
+      <c r="J76" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5269,15 +5652,20 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT fifo)</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT fifo</t>
         </is>
       </c>
-      <c r="H77" s="4" t="inlineStr">
+      <c r="I77" s="4" t="inlineStr">
         <is>
           <t>Config demand_mode = replay</t>
         </is>
       </c>
-      <c r="I77" s="4" t="inlineStr">
+      <c r="J77" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5316,15 +5704,20 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
+          <t>switch (a filled SetupMatrix sheet)</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Routing setup_time_min on every lot</t>
         </is>
       </c>
-      <c r="H78" s="4" t="inlineStr">
+      <c r="I78" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I78" s="4" t="inlineStr">
+      <c r="J78" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5363,15 +5756,20 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Routing setup_time_min on every lot</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr">
+      <c r="I79" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I79" s="4" t="inlineStr">
+      <c r="J79" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5410,15 +5808,20 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Routing setup_time_min on every lot</t>
         </is>
       </c>
-      <c r="H80" s="4" t="inlineStr">
+      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I80" s="4" t="inlineStr">
+      <c r="J80" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5457,15 +5860,20 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
           <t>sheet absent: COPY of Routing setup_time_min on every lot</t>
         </is>
       </c>
-      <c r="H81" s="4" t="inlineStr">
+      <c r="I81" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I81" s="4" t="inlineStr">
+      <c r="J81" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5504,15 +5912,20 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
+          <t>needed (matrix applies only to steps with a family)</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H82" s="4" t="inlineStr">
+      <c r="I82" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I82" s="4" t="inlineStr">
+      <c r="J82" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5551,15 +5964,20 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
           <t>empty text</t>
         </is>
       </c>
-      <c r="H83" s="4" t="inlineStr">
+      <c r="I83" s="4" t="inlineStr">
         <is>
           <t>SetupMatrix sheet present</t>
         </is>
       </c>
-      <c r="I83" s="4" t="inlineStr">
+      <c r="J83" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5598,15 +6016,20 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
+          <t>switch (a value &gt; 0)</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0 = OFF (no breakdowns)</t>
         </is>
       </c>
-      <c r="H84" s="4" t="inlineStr">
+      <c r="I84" s="4" t="inlineStr">
         <is>
           <t>Machines MTBF_hours &gt; 0</t>
         </is>
       </c>
-      <c r="I84" s="4" t="inlineStr">
+      <c r="J84" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5645,15 +6068,20 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
+          <t>needed (blank = repair takes 0 minutes)</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H85" s="4" t="inlineStr">
+      <c r="I85" s="4" t="inlineStr">
         <is>
           <t>Machines MTBF_hours &gt; 0</t>
         </is>
       </c>
-      <c r="I85" s="4" t="inlineStr">
+      <c r="J85" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5692,15 +6120,20 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
           <t>start_qty DEFAULT 0</t>
         </is>
       </c>
-      <c r="H86" s="4" t="inlineStr">
+      <c r="I86" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I86" s="4" t="inlineStr">
+      <c r="J86" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5739,15 +6172,20 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
+          <t>needed (blank = 0)</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
           <t>start_qty DEFAULT 0</t>
         </is>
       </c>
-      <c r="H87" s="4" t="inlineStr">
+      <c r="I87" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I87" s="4" t="inlineStr">
+      <c r="J87" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5786,15 +6224,20 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
           <t>qty DEFAULT 0, issue_step DEFAULT 0, scrap_pct DEFAULT 0</t>
         </is>
       </c>
-      <c r="H88" s="4" t="inlineStr">
+      <c r="I88" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I88" s="4" t="inlineStr">
+      <c r="J88" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5833,15 +6276,20 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
           <t>qty DEFAULT 0, issue_step DEFAULT 0, scrap_pct DEFAULT 0</t>
         </is>
       </c>
-      <c r="H89" s="4" t="inlineStr">
+      <c r="I89" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I89" s="4" t="inlineStr">
+      <c r="J89" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5880,15 +6328,20 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
+          <t>needed (blank = 0)</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
           <t>qty DEFAULT 0, issue_step DEFAULT 0, scrap_pct DEFAULT 0</t>
         </is>
       </c>
-      <c r="H90" s="4" t="inlineStr">
+      <c r="I90" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I90" s="4" t="inlineStr">
+      <c r="J90" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5927,15 +6380,20 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
           <t>qty DEFAULT 0, issue_step DEFAULT 0, scrap_pct DEFAULT 0</t>
         </is>
       </c>
-      <c r="H91" s="4" t="inlineStr">
+      <c r="I91" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I91" s="4" t="inlineStr">
+      <c r="J91" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -5974,15 +6432,20 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
+          <t>optional (DEFAULT 0)</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
           <t>qty DEFAULT 0, issue_step DEFAULT 0, scrap_pct DEFAULT 0</t>
         </is>
       </c>
-      <c r="H92" s="4" t="inlineStr">
+      <c r="I92" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I92" s="4" t="inlineStr">
+      <c r="J92" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6021,15 +6484,20 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
+          <t>switch (boards)</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT off</t>
         </is>
       </c>
-      <c r="H93" s="4" t="inlineStr">
+      <c r="I93" s="4" t="inlineStr">
         <is>
           <t>Config material_mode = boards</t>
         </is>
       </c>
-      <c r="I93" s="4" t="inlineStr">
+      <c r="J93" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6068,15 +6536,20 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
+          <t>needed (blank = 100, no loss)</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 100 = no loss</t>
         </is>
       </c>
-      <c r="H94" s="4" t="inlineStr">
+      <c r="I94" s="4" t="inlineStr">
         <is>
           <t>Config quality_mode = yield</t>
         </is>
       </c>
-      <c r="I94" s="4" t="inlineStr">
+      <c r="J94" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6115,15 +6588,20 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
+          <t>optional</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
           <t>blank or scrap = scrap; rework = one rework pass. Scrapped order pieces get make-up lots, at most 5 per order</t>
         </is>
       </c>
-      <c r="H95" s="4" t="inlineStr">
+      <c r="I95" s="4" t="inlineStr">
         <is>
           <t>Config quality_mode = yield</t>
         </is>
       </c>
-      <c r="I95" s="4" t="inlineStr">
+      <c r="J95" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6162,15 +6640,20 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
+          <t>switch (yield)</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT off</t>
         </is>
       </c>
-      <c r="H96" s="4" t="inlineStr">
+      <c r="I96" s="4" t="inlineStr">
         <is>
           <t>Config quality_mode = yield</t>
         </is>
       </c>
-      <c r="I96" s="4" t="inlineStr">
+      <c r="J96" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6209,15 +6692,20 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
+          <t>switch (a value &gt; 0; or Workers hourly_cost)</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0 = no cost rows</t>
         </is>
       </c>
-      <c r="H97" s="4" t="inlineStr">
+      <c r="I97" s="4" t="inlineStr">
         <is>
           <t>Machines cost_per_hour &gt; 0</t>
         </is>
       </c>
-      <c r="I97" s="4" t="inlineStr">
+      <c r="J97" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6256,15 +6744,20 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
+          <t>switch (a value &gt; 0; or Machines cost_per_hour)</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
           <t>DEFAULT 0</t>
         </is>
       </c>
-      <c r="H98" s="4" t="inlineStr">
+      <c r="I98" s="4" t="inlineStr">
         <is>
           <t>Machines cost_per_hour &gt; 0</t>
         </is>
       </c>
-      <c r="I98" s="4" t="inlineStr">
+      <c r="J98" s="4" t="inlineStr">
         <is>
           <t>tested</t>
         </is>
@@ -6303,15 +6796,20 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
+          <t>switch (Experiment parameter scenario_id names these rows)</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
           <t>rows of other scenario ids are ignored; a scenario id with no rows stops the run</t>
         </is>
       </c>
-      <c r="H99" s="4" t="inlineStr">
+      <c r="I99" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I99" s="4" t="inlineStr">
+      <c r="J99" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6350,15 +6848,20 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
           <t>set / scale / copy / remove; anything else stops the run</t>
         </is>
       </c>
-      <c r="H100" s="4" t="inlineStr">
+      <c r="I100" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I100" s="4" t="inlineStr">
+      <c r="J100" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6397,15 +6900,20 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
           <t>empty or unknown sheet stops the run</t>
         </is>
       </c>
-      <c r="H101" s="4" t="inlineStr">
+      <c r="I101" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I101" s="4" t="inlineStr">
+      <c r="J101" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6444,15 +6952,20 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
           <t>exact id in the first column, prefix* (prefix match; * alone = all rows) or group:X (column resource_group); no match stops the run</t>
         </is>
       </c>
-      <c r="H102" s="4" t="inlineStr">
+      <c r="I102" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I102" s="4" t="inlineStr">
+      <c r="J102" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6491,15 +7004,20 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
+          <t>needed for set / scale</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
           <t>header name; required for set and scale</t>
         </is>
       </c>
-      <c r="H103" s="4" t="inlineStr">
+      <c r="I103" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I103" s="4" t="inlineStr">
+      <c r="J103" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6538,15 +7056,20 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
+          <t>needed for set / scale / copy</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
           <t>set: new value; scale: factor (blank or text cells are skipped); copy: new id (copies linked rows too: Machines -&gt; calendar, alternatives; Workers -&gt; skills, group caps, calendar; Products -&gt; routing, alternatives, BOM); remove: not used (removes linked rows too, Products also its Orders). $p parameter hooks are not built</t>
         </is>
       </c>
-      <c r="H104" s="4" t="inlineStr">
+      <c r="I104" s="4" t="inlineStr">
         <is>
           <t>Experiment parameter scenario_id names rows of the Scenarios sheet</t>
         </is>
       </c>
-      <c r="I104" s="4" t="inlineStr">
+      <c r="J104" s="4" t="inlineStr">
         <is>
           <t>built, not yet tested (test planned Mon 2026-10-26)</t>
         </is>
@@ -6585,15 +7108,20 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
+          <t>not used yet</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
           <t>in the source data; not used by the model yet (staffing_factor_per_machine is used)</t>
         </is>
       </c>
-      <c r="H105" s="4" t="inlineStr">
+      <c r="I105" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I105" s="4" t="inlineStr">
+      <c r="J105" s="4" t="inlineStr">
         <is>
           <t>not used yet</t>
         </is>
@@ -6632,15 +7160,20 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
+          <t>open decision</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
           <t>in the source data; not used by the model yet; open decision whether to apply it (availability comes from MTBF_hours / MTTR_min for now)</t>
         </is>
       </c>
-      <c r="H106" s="4" t="inlineStr">
+      <c r="I106" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I106" s="4" t="inlineStr">
+      <c r="J106" s="4" t="inlineStr">
         <is>
           <t>open decision</t>
         </is>
@@ -6679,15 +7212,20 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
+          <t>not used yet</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
           <t>in the source data; not used by the model yet (cleaning time is inside setup_time_min)</t>
         </is>
       </c>
-      <c r="H107" s="4" t="inlineStr">
+      <c r="I107" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I107" s="4" t="inlineStr">
+      <c r="J107" s="4" t="inlineStr">
         <is>
           <t>not used yet</t>
         </is>
@@ -6726,15 +7264,20 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
+          <t>not used yet</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
           <t>in the source data; not used by the model yet</t>
         </is>
       </c>
-      <c r="H108" s="4" t="inlineStr">
+      <c r="I108" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I108" s="4" t="inlineStr">
+      <c r="J108" s="4" t="inlineStr">
         <is>
           <t>not used yet</t>
         </is>

</xml_diff>